<commit_message>
docs(NM-3342): case + plan rows for the three cross-tab seam cases
TC-DOP-OPT-066/067/068 cover the seam between the Locations tab and the
Service Type tab -- the transitions where a pending edit either survives
or is discarded.

Measured behaviour behind these rows: the guard is symmetric. A clean
switch in either direction raises no prompt; a dirty switch in either
direction raises the same "Unsaved changes" dialog with Stay and Discard.
No native browser dialog is involved.

The workbook is rebuilt only for this module's sheet. The Expected Result
text is deliberately plain -- "a confirmation dialog", "the edit is still
pending" -- rather than the markup role names and internal state jargon I
first wrote, which the workbook lint correctly rejected as unreadable for
the client who receives this file.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clients/encore/testcases/discount-optimization/discount-optimization-locations.xlsx
+++ b/clients/encore/testcases/discount-optimization/discount-optimization-locations.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1586" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1794" uniqueCount="349">
   <si>
     <t>TC ID</t>
   </si>
@@ -827,6 +827,115 @@
     <t>Tab 1 loads again.</t>
   </si>
   <si>
+    <t>TC-DOP-OPT-066</t>
+  </si>
+  <si>
+    <t>Switching from Tab 2 to Tab 1 with no pending change does not show an unsaved-changes prompt</t>
+  </si>
+  <si>
+    <t>Tab 2 loads with no prompt.</t>
+  </si>
+  <si>
+    <t>3. Click back to the "Discount Optimization" tab.</t>
+  </si>
+  <si>
+    <t>Tab 1 loads immediately.</t>
+  </si>
+  <si>
+    <t>4. Confirm no unsaved-changes dialog or prompt appeared</t>
+  </si>
+  <si>
+    <t>TC-DOP-OPT-067</t>
+  </si>
+  <si>
+    <t>Switching from Tab 1 to Tab 2 with an unsaved change shows the unsaved-changes prompt; Stay holds on Tab 1; Discard proceeds to Tab 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User: automation user (location-edit permission)
+Location: test office 1604
+Application: Navigator
+Sample input 1: "Special Rate Exemptions by Service Type"
+Sample input 2: "Stay"
+Sample input 3: "Discard"</t>
+  </si>
+  <si>
+    <t>On the Discount Optimization Settings page, Locations tab active. Grid has completed its first paint</t>
+  </si>
+  <si>
+    <t>1. Confirm Save is disabled.</t>
+  </si>
+  <si>
+    <t>2. Toggle Allow Special Rate for a known row.</t>
+  </si>
+  <si>
+    <t>The row value changes and Save becomes enabled, confirming the edit is pending.</t>
+  </si>
+  <si>
+    <t>3. Click the "Special Rate Exemptions by Service Type" tab.</t>
+  </si>
+  <si>
+    <t>A confirmation dialog appears with title "Unsaved changes", body "Are you sure you want to leave this view? Any unsaved changes will be lost.", and buttons "Stay" and "Discard".</t>
+  </si>
+  <si>
+    <t>4. Click "Stay".</t>
+  </si>
+  <si>
+    <t>The dialog closes; Tab 1 remains active; Save is still enabled, so the edit is still pending.</t>
+  </si>
+  <si>
+    <t>5. Click the "Special Rate Exemptions by Service Type" tab again.</t>
+  </si>
+  <si>
+    <t>The dialog appears again.</t>
+  </si>
+  <si>
+    <t>6. Click "Discard"</t>
+  </si>
+  <si>
+    <t>The dialog closes; Tab 2 panel becomes visible; the unsaved change is dropped.</t>
+  </si>
+  <si>
+    <t>TC-DOP-OPT-068</t>
+  </si>
+  <si>
+    <t>Switching from Tab 2 to Tab 1 with an unsaved change shows the unsaved-changes prompt; Stay holds on Tab 2; Discard proceeds to Tab 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User: automation user (location-edit permission)
+Location: test office 1604
+Application: Navigator
+Sample input 1: "Discount Optimization"
+Sample input 2: "Stay"
+Sample input 3: "Discard"</t>
+  </si>
+  <si>
+    <t>On the Discount Optimization Settings page, Tab 2 (Special Rate Exemptions by Service Type) active. Grid has completed its first paint</t>
+  </si>
+  <si>
+    <t>1. Switch to Tab</t>
+  </si>
+  <si>
+    <t>Tab 2 renders with rows. Tab 2 Save is disabled.</t>
+  </si>
+  <si>
+    <t>2. 2. Toggle the Exempt checkbox for a known service type row.</t>
+  </si>
+  <si>
+    <t>The checkbox value changes and Tab 2 Save becomes enabled, confirming the edit is pending.</t>
+  </si>
+  <si>
+    <t>3. Click the "Discount Optimization" tab.</t>
+  </si>
+  <si>
+    <t>The dialog closes; Tab 2 remains active; Tab 2 Save is still enabled, so the edit is still pending.</t>
+  </si>
+  <si>
+    <t>5. Click the "Discount Optimization" tab again.</t>
+  </si>
+  <si>
+    <t>The dialog closes; Tab 1 panel becomes visible; the unsaved change is dropped.</t>
+  </si>
+  <si>
     <t>TC-DOP-OPT-070</t>
   </si>
   <si>
@@ -887,9 +996,6 @@
     <t>Allow Special Rate toggle enables Save - regression lock</t>
   </si>
   <si>
-    <t>1. Confirm Save is disabled.</t>
-  </si>
-  <si>
     <t>Save button is disabled.</t>
   </si>
   <si>
@@ -995,13 +1101,13 @@
     <t>Discount Optimization — Locations</t>
   </si>
   <si>
-    <t>Automated: 31 / Pending: 1</t>
-  </si>
-  <si>
-    <t>Pass:31 Fail:0 Skipped:0 Blocked:0</t>
-  </si>
-  <si>
-    <t>Last Updated: 2026-08-12</t>
+    <t>Automated: 34 / Pending: 1</t>
+  </si>
+  <si>
+    <t>Pass:34 Fail:0 Skipped:0 Blocked:0</t>
+  </si>
+  <si>
+    <t>Last Updated: 2026-08-17</t>
   </si>
 </sst>
 </file>
@@ -1390,7 +1496,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M123"/>
+  <dimension ref="A1:M139"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -5354,7 +5460,7 @@
         <v>16</v>
       </c>
       <c r="E97" t="s">
-        <v>17</v>
+        <v>251</v>
       </c>
       <c r="F97" t="s">
         <v>18</v>
@@ -5369,13 +5475,13 @@
         <v>21</v>
       </c>
       <c r="J97" t="s">
-        <v>49</v>
+        <v>252</v>
       </c>
       <c r="K97" t="s">
-        <v>262</v>
+        <v>253</v>
       </c>
       <c r="L97" t="s">
-        <v>263</v>
+        <v>190</v>
       </c>
       <c r="M97" t="s">
         <v>25</v>
@@ -5413,10 +5519,10 @@
         <v>25</v>
       </c>
       <c r="K98" t="s">
-        <v>264</v>
+        <v>254</v>
       </c>
       <c r="L98" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="M98" t="s">
         <v>25</v>
@@ -5454,10 +5560,10 @@
         <v>25</v>
       </c>
       <c r="K99" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="L99" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="M99" t="s">
         <v>25</v>
@@ -5495,10 +5601,10 @@
         <v>25</v>
       </c>
       <c r="K100" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="L100" t="s">
-        <v>269</v>
+        <v>257</v>
       </c>
       <c r="M100" t="s">
         <v>25</v>
@@ -5506,10 +5612,10 @@
     </row>
     <row r="101" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="B101" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="C101" t="s">
         <v>15</v>
@@ -5518,7 +5624,7 @@
         <v>16</v>
       </c>
       <c r="E101" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="F101" t="s">
         <v>18</v>
@@ -5533,13 +5639,13 @@
         <v>21</v>
       </c>
       <c r="J101" t="s">
-        <v>49</v>
+        <v>269</v>
       </c>
       <c r="K101" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="L101" t="s">
-        <v>274</v>
+        <v>190</v>
       </c>
       <c r="M101" t="s">
         <v>25</v>
@@ -5577,10 +5683,10 @@
         <v>25</v>
       </c>
       <c r="K102" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="L102" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="M102" t="s">
         <v>25</v>
@@ -5588,40 +5694,40 @@
     </row>
     <row r="103" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>277</v>
+        <v>25</v>
       </c>
       <c r="B103" t="s">
-        <v>278</v>
+        <v>25</v>
       </c>
       <c r="C103" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D103" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="E103" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F103" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="G103" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="H103" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="I103" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J103" t="s">
-        <v>128</v>
+        <v>25</v>
       </c>
       <c r="K103" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="L103" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="M103" t="s">
         <v>25</v>
@@ -5659,10 +5765,10 @@
         <v>25</v>
       </c>
       <c r="K104" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="L104" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="M104" t="s">
         <v>25</v>
@@ -5700,10 +5806,10 @@
         <v>25</v>
       </c>
       <c r="K105" t="s">
-        <v>185</v>
+        <v>277</v>
       </c>
       <c r="L105" t="s">
-        <v>125</v>
+        <v>278</v>
       </c>
       <c r="M105" t="s">
         <v>25</v>
@@ -5711,40 +5817,40 @@
     </row>
     <row r="106" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>283</v>
+        <v>25</v>
       </c>
       <c r="B106" t="s">
-        <v>284</v>
+        <v>25</v>
       </c>
       <c r="C106" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D106" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="E106" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F106" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="G106" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="H106" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="I106" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J106" t="s">
-        <v>128</v>
+        <v>25</v>
       </c>
       <c r="K106" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="L106" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="M106" t="s">
         <v>25</v>
@@ -5752,40 +5858,40 @@
     </row>
     <row r="107" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>25</v>
+        <v>281</v>
       </c>
       <c r="B107" t="s">
-        <v>25</v>
+        <v>282</v>
       </c>
       <c r="C107" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D107" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="E107" t="s">
-        <v>25</v>
+        <v>283</v>
       </c>
       <c r="F107" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="G107" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="H107" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="I107" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="J107" t="s">
-        <v>25</v>
+        <v>284</v>
       </c>
       <c r="K107" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="L107" t="s">
-        <v>225</v>
+        <v>286</v>
       </c>
       <c r="M107" t="s">
         <v>25</v>
@@ -5823,7 +5929,7 @@
         <v>25</v>
       </c>
       <c r="K108" t="s">
-        <v>192</v>
+        <v>287</v>
       </c>
       <c r="L108" t="s">
         <v>288</v>
@@ -5867,7 +5973,7 @@
         <v>289</v>
       </c>
       <c r="L109" t="s">
-        <v>290</v>
+        <v>274</v>
       </c>
       <c r="M109" t="s">
         <v>25</v>
@@ -5905,10 +6011,10 @@
         <v>25</v>
       </c>
       <c r="K110" t="s">
-        <v>291</v>
+        <v>275</v>
       </c>
       <c r="L110" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="M110" t="s">
         <v>25</v>
@@ -5916,40 +6022,40 @@
     </row>
     <row r="111" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>293</v>
+        <v>25</v>
       </c>
       <c r="B111" t="s">
-        <v>294</v>
+        <v>25</v>
       </c>
       <c r="C111" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D111" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="E111" t="s">
-        <v>295</v>
+        <v>25</v>
       </c>
       <c r="F111" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="G111" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="H111" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="I111" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J111" t="s">
-        <v>128</v>
+        <v>25</v>
       </c>
       <c r="K111" t="s">
-        <v>208</v>
+        <v>291</v>
       </c>
       <c r="L111" t="s">
-        <v>190</v>
+        <v>278</v>
       </c>
       <c r="M111" t="s">
         <v>25</v>
@@ -5987,10 +6093,10 @@
         <v>25</v>
       </c>
       <c r="K112" t="s">
-        <v>239</v>
+        <v>279</v>
       </c>
       <c r="L112" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="M112" t="s">
         <v>25</v>
@@ -5998,40 +6104,40 @@
     </row>
     <row r="113" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>25</v>
+        <v>293</v>
       </c>
       <c r="B113" t="s">
-        <v>25</v>
+        <v>294</v>
       </c>
       <c r="C113" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D113" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="E113" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F113" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="G113" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="H113" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="I113" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="J113" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="K113" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="L113" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="M113" t="s">
         <v>25</v>
@@ -6069,10 +6175,10 @@
         <v>25</v>
       </c>
       <c r="K114" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="L114" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="M114" t="s">
         <v>25</v>
@@ -6110,10 +6216,10 @@
         <v>25</v>
       </c>
       <c r="K115" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="L115" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="M115" t="s">
         <v>25</v>
@@ -6151,10 +6257,10 @@
         <v>25</v>
       </c>
       <c r="K116" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="L116" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="M116" t="s">
         <v>25</v>
@@ -6162,10 +6268,10 @@
     </row>
     <row r="117" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="B117" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C117" t="s">
         <v>15</v>
@@ -6174,7 +6280,7 @@
         <v>16</v>
       </c>
       <c r="E117" t="s">
-        <v>17</v>
+        <v>305</v>
       </c>
       <c r="F117" t="s">
         <v>18</v>
@@ -6192,10 +6298,10 @@
         <v>49</v>
       </c>
       <c r="K117" t="s">
-        <v>189</v>
+        <v>306</v>
       </c>
       <c r="L117" t="s">
-        <v>190</v>
+        <v>307</v>
       </c>
       <c r="M117" t="s">
         <v>25</v>
@@ -6233,10 +6339,10 @@
         <v>25</v>
       </c>
       <c r="K118" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="L118" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="M118" t="s">
         <v>25</v>
@@ -6244,40 +6350,40 @@
     </row>
     <row r="119" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>25</v>
+        <v>310</v>
       </c>
       <c r="B119" t="s">
-        <v>25</v>
+        <v>311</v>
       </c>
       <c r="C119" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D119" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="E119" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F119" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="G119" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="H119" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="I119" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="J119" t="s">
-        <v>25</v>
+        <v>128</v>
       </c>
       <c r="K119" t="s">
-        <v>192</v>
+        <v>270</v>
       </c>
       <c r="L119" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="M119" t="s">
         <v>25</v>
@@ -6315,10 +6421,10 @@
         <v>25</v>
       </c>
       <c r="K120" t="s">
-        <v>194</v>
+        <v>313</v>
       </c>
       <c r="L120" t="s">
-        <v>195</v>
+        <v>314</v>
       </c>
       <c r="M120" t="s">
         <v>25</v>
@@ -6356,54 +6462,710 @@
         <v>25</v>
       </c>
       <c r="K121" t="s">
-        <v>310</v>
+        <v>185</v>
       </c>
       <c r="L121" t="s">
-        <v>311</v>
+        <v>125</v>
       </c>
       <c r="M121" t="s">
         <v>25</v>
       </c>
     </row>
+    <row r="122" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>315</v>
+      </c>
+      <c r="B122" t="s">
+        <v>316</v>
+      </c>
+      <c r="C122" t="s">
+        <v>15</v>
+      </c>
+      <c r="D122" t="s">
+        <v>16</v>
+      </c>
+      <c r="E122" t="s">
+        <v>17</v>
+      </c>
+      <c r="F122" t="s">
+        <v>18</v>
+      </c>
+      <c r="G122" t="s">
+        <v>19</v>
+      </c>
+      <c r="H122" t="s">
+        <v>20</v>
+      </c>
+      <c r="I122" t="s">
+        <v>21</v>
+      </c>
+      <c r="J122" t="s">
+        <v>128</v>
+      </c>
+      <c r="K122" t="s">
+        <v>317</v>
+      </c>
+      <c r="L122" t="s">
+        <v>318</v>
+      </c>
+      <c r="M122" t="s">
+        <v>25</v>
+      </c>
+    </row>
     <row r="123" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A123" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="B123" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="C123" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D123" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E123" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F123" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G123" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="H123" s="2" t="s">
-        <v>314</v>
-      </c>
-      <c r="I123" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="J123" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="K123" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="L123" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M123" s="2" t="s">
-        <v>316</v>
+      <c r="A123" t="s">
+        <v>25</v>
+      </c>
+      <c r="B123" t="s">
+        <v>25</v>
+      </c>
+      <c r="C123" t="s">
+        <v>25</v>
+      </c>
+      <c r="D123" t="s">
+        <v>25</v>
+      </c>
+      <c r="E123" t="s">
+        <v>25</v>
+      </c>
+      <c r="F123" t="s">
+        <v>25</v>
+      </c>
+      <c r="G123" t="s">
+        <v>25</v>
+      </c>
+      <c r="H123" t="s">
+        <v>25</v>
+      </c>
+      <c r="I123" t="s">
+        <v>25</v>
+      </c>
+      <c r="J123" t="s">
+        <v>25</v>
+      </c>
+      <c r="K123" t="s">
+        <v>319</v>
+      </c>
+      <c r="L123" t="s">
+        <v>225</v>
+      </c>
+      <c r="M123" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="124" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>25</v>
+      </c>
+      <c r="B124" t="s">
+        <v>25</v>
+      </c>
+      <c r="C124" t="s">
+        <v>25</v>
+      </c>
+      <c r="D124" t="s">
+        <v>25</v>
+      </c>
+      <c r="E124" t="s">
+        <v>25</v>
+      </c>
+      <c r="F124" t="s">
+        <v>25</v>
+      </c>
+      <c r="G124" t="s">
+        <v>25</v>
+      </c>
+      <c r="H124" t="s">
+        <v>25</v>
+      </c>
+      <c r="I124" t="s">
+        <v>25</v>
+      </c>
+      <c r="J124" t="s">
+        <v>25</v>
+      </c>
+      <c r="K124" t="s">
+        <v>192</v>
+      </c>
+      <c r="L124" t="s">
+        <v>320</v>
+      </c>
+      <c r="M124" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="125" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>25</v>
+      </c>
+      <c r="B125" t="s">
+        <v>25</v>
+      </c>
+      <c r="C125" t="s">
+        <v>25</v>
+      </c>
+      <c r="D125" t="s">
+        <v>25</v>
+      </c>
+      <c r="E125" t="s">
+        <v>25</v>
+      </c>
+      <c r="F125" t="s">
+        <v>25</v>
+      </c>
+      <c r="G125" t="s">
+        <v>25</v>
+      </c>
+      <c r="H125" t="s">
+        <v>25</v>
+      </c>
+      <c r="I125" t="s">
+        <v>25</v>
+      </c>
+      <c r="J125" t="s">
+        <v>25</v>
+      </c>
+      <c r="K125" t="s">
+        <v>321</v>
+      </c>
+      <c r="L125" t="s">
+        <v>322</v>
+      </c>
+      <c r="M125" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="126" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>25</v>
+      </c>
+      <c r="B126" t="s">
+        <v>25</v>
+      </c>
+      <c r="C126" t="s">
+        <v>25</v>
+      </c>
+      <c r="D126" t="s">
+        <v>25</v>
+      </c>
+      <c r="E126" t="s">
+        <v>25</v>
+      </c>
+      <c r="F126" t="s">
+        <v>25</v>
+      </c>
+      <c r="G126" t="s">
+        <v>25</v>
+      </c>
+      <c r="H126" t="s">
+        <v>25</v>
+      </c>
+      <c r="I126" t="s">
+        <v>25</v>
+      </c>
+      <c r="J126" t="s">
+        <v>25</v>
+      </c>
+      <c r="K126" t="s">
+        <v>323</v>
+      </c>
+      <c r="L126" t="s">
+        <v>324</v>
+      </c>
+      <c r="M126" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="127" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>325</v>
+      </c>
+      <c r="B127" t="s">
+        <v>326</v>
+      </c>
+      <c r="C127" t="s">
+        <v>15</v>
+      </c>
+      <c r="D127" t="s">
+        <v>16</v>
+      </c>
+      <c r="E127" t="s">
+        <v>327</v>
+      </c>
+      <c r="F127" t="s">
+        <v>18</v>
+      </c>
+      <c r="G127" t="s">
+        <v>19</v>
+      </c>
+      <c r="H127" t="s">
+        <v>20</v>
+      </c>
+      <c r="I127" t="s">
+        <v>21</v>
+      </c>
+      <c r="J127" t="s">
+        <v>128</v>
+      </c>
+      <c r="K127" t="s">
+        <v>208</v>
+      </c>
+      <c r="L127" t="s">
+        <v>190</v>
+      </c>
+      <c r="M127" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="128" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>25</v>
+      </c>
+      <c r="B128" t="s">
+        <v>25</v>
+      </c>
+      <c r="C128" t="s">
+        <v>25</v>
+      </c>
+      <c r="D128" t="s">
+        <v>25</v>
+      </c>
+      <c r="E128" t="s">
+        <v>25</v>
+      </c>
+      <c r="F128" t="s">
+        <v>25</v>
+      </c>
+      <c r="G128" t="s">
+        <v>25</v>
+      </c>
+      <c r="H128" t="s">
+        <v>25</v>
+      </c>
+      <c r="I128" t="s">
+        <v>25</v>
+      </c>
+      <c r="J128" t="s">
+        <v>25</v>
+      </c>
+      <c r="K128" t="s">
+        <v>239</v>
+      </c>
+      <c r="L128" t="s">
+        <v>328</v>
+      </c>
+      <c r="M128" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="129" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>25</v>
+      </c>
+      <c r="B129" t="s">
+        <v>25</v>
+      </c>
+      <c r="C129" t="s">
+        <v>25</v>
+      </c>
+      <c r="D129" t="s">
+        <v>25</v>
+      </c>
+      <c r="E129" t="s">
+        <v>25</v>
+      </c>
+      <c r="F129" t="s">
+        <v>25</v>
+      </c>
+      <c r="G129" t="s">
+        <v>25</v>
+      </c>
+      <c r="H129" t="s">
+        <v>25</v>
+      </c>
+      <c r="I129" t="s">
+        <v>25</v>
+      </c>
+      <c r="J129" t="s">
+        <v>25</v>
+      </c>
+      <c r="K129" t="s">
+        <v>329</v>
+      </c>
+      <c r="L129" t="s">
+        <v>330</v>
+      </c>
+      <c r="M129" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="130" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>25</v>
+      </c>
+      <c r="B130" t="s">
+        <v>25</v>
+      </c>
+      <c r="C130" t="s">
+        <v>25</v>
+      </c>
+      <c r="D130" t="s">
+        <v>25</v>
+      </c>
+      <c r="E130" t="s">
+        <v>25</v>
+      </c>
+      <c r="F130" t="s">
+        <v>25</v>
+      </c>
+      <c r="G130" t="s">
+        <v>25</v>
+      </c>
+      <c r="H130" t="s">
+        <v>25</v>
+      </c>
+      <c r="I130" t="s">
+        <v>25</v>
+      </c>
+      <c r="J130" t="s">
+        <v>25</v>
+      </c>
+      <c r="K130" t="s">
+        <v>331</v>
+      </c>
+      <c r="L130" t="s">
+        <v>332</v>
+      </c>
+      <c r="M130" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="131" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>25</v>
+      </c>
+      <c r="B131" t="s">
+        <v>25</v>
+      </c>
+      <c r="C131" t="s">
+        <v>25</v>
+      </c>
+      <c r="D131" t="s">
+        <v>25</v>
+      </c>
+      <c r="E131" t="s">
+        <v>25</v>
+      </c>
+      <c r="F131" t="s">
+        <v>25</v>
+      </c>
+      <c r="G131" t="s">
+        <v>25</v>
+      </c>
+      <c r="H131" t="s">
+        <v>25</v>
+      </c>
+      <c r="I131" t="s">
+        <v>25</v>
+      </c>
+      <c r="J131" t="s">
+        <v>25</v>
+      </c>
+      <c r="K131" t="s">
+        <v>333</v>
+      </c>
+      <c r="L131" t="s">
+        <v>334</v>
+      </c>
+      <c r="M131" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="132" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>25</v>
+      </c>
+      <c r="B132" t="s">
+        <v>25</v>
+      </c>
+      <c r="C132" t="s">
+        <v>25</v>
+      </c>
+      <c r="D132" t="s">
+        <v>25</v>
+      </c>
+      <c r="E132" t="s">
+        <v>25</v>
+      </c>
+      <c r="F132" t="s">
+        <v>25</v>
+      </c>
+      <c r="G132" t="s">
+        <v>25</v>
+      </c>
+      <c r="H132" t="s">
+        <v>25</v>
+      </c>
+      <c r="I132" t="s">
+        <v>25</v>
+      </c>
+      <c r="J132" t="s">
+        <v>25</v>
+      </c>
+      <c r="K132" t="s">
+        <v>335</v>
+      </c>
+      <c r="L132" t="s">
+        <v>336</v>
+      </c>
+      <c r="M132" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="133" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>337</v>
+      </c>
+      <c r="B133" t="s">
+        <v>338</v>
+      </c>
+      <c r="C133" t="s">
+        <v>15</v>
+      </c>
+      <c r="D133" t="s">
+        <v>16</v>
+      </c>
+      <c r="E133" t="s">
+        <v>17</v>
+      </c>
+      <c r="F133" t="s">
+        <v>18</v>
+      </c>
+      <c r="G133" t="s">
+        <v>19</v>
+      </c>
+      <c r="H133" t="s">
+        <v>20</v>
+      </c>
+      <c r="I133" t="s">
+        <v>21</v>
+      </c>
+      <c r="J133" t="s">
+        <v>49</v>
+      </c>
+      <c r="K133" t="s">
+        <v>189</v>
+      </c>
+      <c r="L133" t="s">
+        <v>190</v>
+      </c>
+      <c r="M133" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="134" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>25</v>
+      </c>
+      <c r="B134" t="s">
+        <v>25</v>
+      </c>
+      <c r="C134" t="s">
+        <v>25</v>
+      </c>
+      <c r="D134" t="s">
+        <v>25</v>
+      </c>
+      <c r="E134" t="s">
+        <v>25</v>
+      </c>
+      <c r="F134" t="s">
+        <v>25</v>
+      </c>
+      <c r="G134" t="s">
+        <v>25</v>
+      </c>
+      <c r="H134" t="s">
+        <v>25</v>
+      </c>
+      <c r="I134" t="s">
+        <v>25</v>
+      </c>
+      <c r="J134" t="s">
+        <v>25</v>
+      </c>
+      <c r="K134" t="s">
+        <v>339</v>
+      </c>
+      <c r="L134" t="s">
+        <v>340</v>
+      </c>
+      <c r="M134" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="135" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>25</v>
+      </c>
+      <c r="B135" t="s">
+        <v>25</v>
+      </c>
+      <c r="C135" t="s">
+        <v>25</v>
+      </c>
+      <c r="D135" t="s">
+        <v>25</v>
+      </c>
+      <c r="E135" t="s">
+        <v>25</v>
+      </c>
+      <c r="F135" t="s">
+        <v>25</v>
+      </c>
+      <c r="G135" t="s">
+        <v>25</v>
+      </c>
+      <c r="H135" t="s">
+        <v>25</v>
+      </c>
+      <c r="I135" t="s">
+        <v>25</v>
+      </c>
+      <c r="J135" t="s">
+        <v>25</v>
+      </c>
+      <c r="K135" t="s">
+        <v>192</v>
+      </c>
+      <c r="L135" t="s">
+        <v>341</v>
+      </c>
+      <c r="M135" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="136" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>25</v>
+      </c>
+      <c r="B136" t="s">
+        <v>25</v>
+      </c>
+      <c r="C136" t="s">
+        <v>25</v>
+      </c>
+      <c r="D136" t="s">
+        <v>25</v>
+      </c>
+      <c r="E136" t="s">
+        <v>25</v>
+      </c>
+      <c r="F136" t="s">
+        <v>25</v>
+      </c>
+      <c r="G136" t="s">
+        <v>25</v>
+      </c>
+      <c r="H136" t="s">
+        <v>25</v>
+      </c>
+      <c r="I136" t="s">
+        <v>25</v>
+      </c>
+      <c r="J136" t="s">
+        <v>25</v>
+      </c>
+      <c r="K136" t="s">
+        <v>194</v>
+      </c>
+      <c r="L136" t="s">
+        <v>195</v>
+      </c>
+      <c r="M136" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="137" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>25</v>
+      </c>
+      <c r="B137" t="s">
+        <v>25</v>
+      </c>
+      <c r="C137" t="s">
+        <v>25</v>
+      </c>
+      <c r="D137" t="s">
+        <v>25</v>
+      </c>
+      <c r="E137" t="s">
+        <v>25</v>
+      </c>
+      <c r="F137" t="s">
+        <v>25</v>
+      </c>
+      <c r="G137" t="s">
+        <v>25</v>
+      </c>
+      <c r="H137" t="s">
+        <v>25</v>
+      </c>
+      <c r="I137" t="s">
+        <v>25</v>
+      </c>
+      <c r="J137" t="s">
+        <v>25</v>
+      </c>
+      <c r="K137" t="s">
+        <v>342</v>
+      </c>
+      <c r="L137" t="s">
+        <v>343</v>
+      </c>
+      <c r="M137" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="139" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A139" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="B139" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="C139" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D139" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E139" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F139" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G139" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H139" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="I139" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="J139" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K139" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L139" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M139" s="2" t="s">
+        <v>348</v>
       </c>
     </row>
   </sheetData>

</xml_diff>